<commit_message>
First run of stockpile build implementation based on APS transactions. Next steps: update stockpile grades by payload grades during the build process, add more controls on stockpile states (build, reclaim, off, auto - only needs an input for reclaim threshold and build can be decided based on APS transactions)
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/output/processed_aps_transactions.xlsx
+++ b/blendmaster_backend_OOP/output/processed_aps_transactions.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\BlendMaster\blendmaster_backend_OOP\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94380A8-1A21-464B-A6E4-0766C3DAC76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36A0BB5-F5CB-451E-87F2-29072224AC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$1161</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -282,7 +285,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -339,7 +342,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -44770,6 +44773,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L1161" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>